<commit_message>
Update Dia-Mes template for haircut management
</commit_message>
<xml_diff>
--- a/templates/Dia-Mes-template.xlsx
+++ b/templates/Dia-Mes-template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thelu\OneDrive\Desktop\The Luxe\2025\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Brian\Documents\TheLuxe\Desarrollo\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F22C6C52-5377-427C-933F-F524A34734FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55BD89A0-FBBC-4541-BAB1-E2227A111309}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{D720BB1E-C668-445F-BB14-D44A68D749F2}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" activeTab="1" xr2:uid="{D720BB1E-C668-445F-BB14-D44A68D749F2}"/>
   </bookViews>
   <sheets>
     <sheet name="Barberos" sheetId="1" r:id="rId1"/>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="27">
   <si>
     <t>Nombre</t>
   </si>
@@ -69,9 +69,6 @@
   </si>
   <si>
     <t>MP</t>
-  </si>
-  <si>
-    <t>The Luxe</t>
   </si>
   <si>
     <t>Fecha:</t>
@@ -113,34 +110,37 @@
     <t>Caja Inicial:</t>
   </si>
   <si>
-    <t>Comisión Barberos</t>
-  </si>
-  <si>
-    <t>Ciro</t>
-  </si>
-  <si>
-    <t>Valentin</t>
-  </si>
-  <si>
-    <t>Joel</t>
-  </si>
-  <si>
-    <t>Matias</t>
-  </si>
-  <si>
-    <t>Braian</t>
-  </si>
-  <si>
-    <t>Julian</t>
-  </si>
-  <si>
     <t>Aclaracion:</t>
   </si>
   <si>
-    <t>Fabricio</t>
+    <t>Barbero1</t>
   </si>
   <si>
-    <t>Bautista</t>
+    <t>Barbero2</t>
+  </si>
+  <si>
+    <t>Barbero3</t>
+  </si>
+  <si>
+    <t>Barbero4</t>
+  </si>
+  <si>
+    <t>Barbero5</t>
+  </si>
+  <si>
+    <t>Barbero6</t>
+  </si>
+  <si>
+    <t>Barbero7</t>
+  </si>
+  <si>
+    <t>Barbero8</t>
+  </si>
+  <si>
+    <t>BARBERIA</t>
+  </si>
+  <si>
+    <t>Comisión Barberos(%)</t>
   </si>
 </sst>
 </file>
@@ -417,65 +417,65 @@
     <xf numFmtId="16" fontId="2" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -759,9 +759,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -799,7 +799,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -905,7 +905,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1047,7 +1047,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1057,67 +1057,68 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{029BBDA5-212E-4FEE-AF16-2002A17AC1B9}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:AJ40"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.21875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.1796875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="10.6328125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="8.54296875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="4.7265625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="7.1796875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="10.6328125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="8.54296875" style="1" customWidth="1"/>
-    <col min="8" max="8" width="4.6328125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="7.1796875" style="1" customWidth="1"/>
-    <col min="10" max="10" width="10.6328125" style="1" customWidth="1"/>
-    <col min="11" max="11" width="8.54296875" style="1" customWidth="1"/>
-    <col min="12" max="12" width="4.6328125" style="1" customWidth="1"/>
-    <col min="13" max="13" width="7.1796875" style="1" customWidth="1"/>
-    <col min="14" max="14" width="10.6328125" style="1" customWidth="1"/>
-    <col min="15" max="15" width="8.54296875" style="1" customWidth="1"/>
-    <col min="16" max="16" width="4.6328125" style="1" customWidth="1"/>
-    <col min="17" max="17" width="7.1796875" style="1" customWidth="1"/>
-    <col min="18" max="18" width="10.6328125" style="1" customWidth="1"/>
-    <col min="19" max="19" width="8.54296875" style="1" customWidth="1"/>
-    <col min="20" max="20" width="4.6328125" style="1" customWidth="1"/>
-    <col min="21" max="21" width="7.1796875" style="1" customWidth="1"/>
-    <col min="22" max="22" width="10.6328125" style="1" customWidth="1"/>
-    <col min="23" max="23" width="8.54296875" style="1" customWidth="1"/>
-    <col min="24" max="24" width="4.6328125" style="1" customWidth="1"/>
-    <col min="25" max="25" width="7.1796875" style="1" customWidth="1"/>
-    <col min="26" max="26" width="10.6328125" style="1" customWidth="1"/>
-    <col min="27" max="27" width="8.54296875" style="1" customWidth="1"/>
-    <col min="28" max="28" width="4.6328125" style="1" customWidth="1"/>
-    <col min="29" max="29" width="7.1796875" style="1" customWidth="1"/>
-    <col min="30" max="30" width="10.6328125" style="1" customWidth="1"/>
-    <col min="31" max="31" width="8.54296875" style="1" customWidth="1"/>
-    <col min="32" max="32" width="4.54296875" style="1" customWidth="1"/>
-    <col min="33" max="33" width="7.1796875" style="1" customWidth="1"/>
-    <col min="34" max="35" width="14.7265625" style="1" customWidth="1"/>
-    <col min="36" max="36" width="4.7265625" style="1" customWidth="1"/>
-    <col min="37" max="16384" width="9.1796875" style="1"/>
+    <col min="1" max="1" width="7.21875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="10.6640625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="8.5546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="4.77734375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="7.21875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="10.6640625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="8.5546875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="4.6640625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="7.21875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="10.6640625" style="1" customWidth="1"/>
+    <col min="11" max="11" width="8.5546875" style="1" customWidth="1"/>
+    <col min="12" max="12" width="6.6640625" style="1" customWidth="1"/>
+    <col min="13" max="13" width="7.21875" style="1" customWidth="1"/>
+    <col min="14" max="14" width="10.6640625" style="1" customWidth="1"/>
+    <col min="15" max="15" width="8.5546875" style="1" customWidth="1"/>
+    <col min="16" max="16" width="4.6640625" style="1" customWidth="1"/>
+    <col min="17" max="17" width="7.21875" style="1" customWidth="1"/>
+    <col min="18" max="18" width="10.6640625" style="1" customWidth="1"/>
+    <col min="19" max="19" width="8.5546875" style="1" customWidth="1"/>
+    <col min="20" max="20" width="4.6640625" style="1" customWidth="1"/>
+    <col min="21" max="21" width="7.21875" style="1" customWidth="1"/>
+    <col min="22" max="22" width="10.6640625" style="1" customWidth="1"/>
+    <col min="23" max="23" width="8.5546875" style="1" customWidth="1"/>
+    <col min="24" max="24" width="4.6640625" style="1" customWidth="1"/>
+    <col min="25" max="25" width="7.21875" style="1" customWidth="1"/>
+    <col min="26" max="26" width="10.6640625" style="1" customWidth="1"/>
+    <col min="27" max="27" width="8.5546875" style="1" customWidth="1"/>
+    <col min="28" max="28" width="4.6640625" style="1" customWidth="1"/>
+    <col min="29" max="29" width="7.21875" style="1" customWidth="1"/>
+    <col min="30" max="30" width="10.6640625" style="1" customWidth="1"/>
+    <col min="31" max="31" width="8.5546875" style="1" customWidth="1"/>
+    <col min="32" max="32" width="4.5546875" style="1" customWidth="1"/>
+    <col min="33" max="33" width="7.21875" style="1" customWidth="1"/>
+    <col min="34" max="34" width="14.77734375" style="1" customWidth="1"/>
+    <col min="35" max="35" width="5.5546875" style="1" customWidth="1"/>
+    <col min="36" max="36" width="4.77734375" style="1" customWidth="1"/>
+    <col min="37" max="16384" width="9.21875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12"/>
       <c r="B1" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" s="13"/>
+      <c r="D1" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="13"/>
-      <c r="D1" s="29" t="s">
-        <v>4</v>
-      </c>
-      <c r="E1" s="30"/>
+      <c r="E1" s="41"/>
       <c r="F1" s="26"/>
-      <c r="G1" s="39" t="s">
-        <v>16</v>
-      </c>
-      <c r="H1" s="39"/>
-      <c r="I1" s="40"/>
-      <c r="J1" s="41"/>
-      <c r="K1" s="42" t="s">
-        <v>17</v>
-      </c>
-      <c r="L1" s="43"/>
+      <c r="G1" s="35" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1" s="35"/>
+      <c r="I1" s="36"/>
+      <c r="J1" s="37"/>
+      <c r="K1" s="38" t="s">
+        <v>26</v>
+      </c>
+      <c r="L1" s="39"/>
       <c r="M1" s="20">
         <v>50</v>
       </c>
@@ -1133,9 +1134,9 @@
       <c r="W1" s="5"/>
       <c r="X1" s="5"/>
     </row>
-    <row r="2" spans="1:36" s="11" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" s="11" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B2" s="10" t="s">
         <v>0</v>
@@ -1147,7 +1148,7 @@
         <v>2</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F2" s="10" t="s">
         <v>0</v>
@@ -1159,7 +1160,7 @@
         <v>2</v>
       </c>
       <c r="I2" s="10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J2" s="10" t="s">
         <v>0</v>
@@ -1171,7 +1172,7 @@
         <v>2</v>
       </c>
       <c r="M2" s="10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="N2" s="10" t="s">
         <v>0</v>
@@ -1183,7 +1184,7 @@
         <v>2</v>
       </c>
       <c r="Q2" s="10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="R2" s="10" t="s">
         <v>0</v>
@@ -1195,7 +1196,7 @@
         <v>2</v>
       </c>
       <c r="U2" s="10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="V2" s="10" t="s">
         <v>0</v>
@@ -1207,7 +1208,7 @@
         <v>2</v>
       </c>
       <c r="Y2" s="10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="Z2" s="10" t="s">
         <v>0</v>
@@ -1219,7 +1220,7 @@
         <v>2</v>
       </c>
       <c r="AC2" s="10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="AD2" s="10" t="s">
         <v>0</v>
@@ -1231,7 +1232,7 @@
         <v>2</v>
       </c>
       <c r="AG2" s="10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="AH2" s="10" t="s">
         <v>0</v>
@@ -1243,63 +1244,63 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="9"/>
       <c r="B3" s="6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C3" s="9"/>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
       <c r="F3" s="6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G3" s="9"/>
       <c r="H3" s="9"/>
       <c r="I3" s="9"/>
       <c r="J3" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K3" s="9"/>
       <c r="L3" s="9"/>
       <c r="M3" s="9"/>
       <c r="N3" s="6" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="O3" s="9"/>
       <c r="P3" s="9"/>
       <c r="Q3" s="9"/>
       <c r="R3" s="6" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="S3" s="9"/>
       <c r="T3" s="9"/>
       <c r="U3" s="9"/>
       <c r="V3" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="W3" s="9"/>
       <c r="X3" s="9"/>
       <c r="Y3" s="9"/>
       <c r="Z3" s="6" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="AA3" s="9"/>
       <c r="AB3" s="9"/>
       <c r="AC3" s="9"/>
       <c r="AD3" s="6" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="AE3" s="9"/>
       <c r="AF3" s="9"/>
       <c r="AG3" s="9"/>
       <c r="AH3" s="6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="AI3" s="9"/>
       <c r="AJ3" s="9"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="21"/>
       <c r="B4" s="22"/>
       <c r="C4" s="17"/>
@@ -1337,7 +1338,7 @@
       <c r="AI4" s="17"/>
       <c r="AJ4" s="3"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
       <c r="B5" s="22"/>
       <c r="C5" s="17"/>
@@ -1375,7 +1376,7 @@
       <c r="AI5" s="17"/>
       <c r="AJ5" s="3"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="3"/>
       <c r="B6" s="22"/>
       <c r="C6" s="17"/>
@@ -1413,7 +1414,7 @@
       <c r="AI6" s="17"/>
       <c r="AJ6" s="3"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="3"/>
       <c r="B7" s="22"/>
       <c r="C7" s="17"/>
@@ -1451,7 +1452,7 @@
       <c r="AI7" s="17"/>
       <c r="AJ7" s="3"/>
     </row>
-    <row r="8" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A8" s="3"/>
       <c r="B8" s="22"/>
       <c r="C8" s="17"/>
@@ -1489,7 +1490,7 @@
       <c r="AI8" s="17"/>
       <c r="AJ8" s="3"/>
     </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A9" s="3"/>
       <c r="B9" s="22"/>
       <c r="C9" s="17"/>
@@ -1527,7 +1528,7 @@
       <c r="AI9" s="17"/>
       <c r="AJ9" s="3"/>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A10" s="3"/>
       <c r="B10" s="22"/>
       <c r="C10" s="17"/>
@@ -1565,7 +1566,7 @@
       <c r="AI10" s="17"/>
       <c r="AJ10" s="3"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="3"/>
       <c r="B11" s="22"/>
       <c r="C11" s="17"/>
@@ -1603,7 +1604,7 @@
       <c r="AI11" s="17"/>
       <c r="AJ11" s="3"/>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="3"/>
       <c r="B12" s="22"/>
       <c r="C12" s="17"/>
@@ -1641,7 +1642,7 @@
       <c r="AI12" s="17"/>
       <c r="AJ12" s="3"/>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="3"/>
       <c r="B13" s="22"/>
       <c r="C13" s="17"/>
@@ -1679,7 +1680,7 @@
       <c r="AI13" s="17"/>
       <c r="AJ13" s="3"/>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="3"/>
       <c r="B14" s="22"/>
       <c r="C14" s="17"/>
@@ -1717,7 +1718,7 @@
       <c r="AI14" s="17"/>
       <c r="AJ14" s="3"/>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="3"/>
       <c r="B15" s="22"/>
       <c r="C15" s="17"/>
@@ -1755,7 +1756,7 @@
       <c r="AI15" s="17"/>
       <c r="AJ15" s="3"/>
     </row>
-    <row r="16" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A16" s="3"/>
       <c r="B16" s="22"/>
       <c r="C16" s="17"/>
@@ -1793,7 +1794,7 @@
       <c r="AI16" s="17"/>
       <c r="AJ16" s="3"/>
     </row>
-    <row r="17" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A17" s="3"/>
       <c r="B17" s="22"/>
       <c r="C17" s="17"/>
@@ -1831,7 +1832,7 @@
       <c r="AI17" s="17"/>
       <c r="AJ17" s="3"/>
     </row>
-    <row r="18" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A18" s="3"/>
       <c r="B18" s="22"/>
       <c r="C18" s="17"/>
@@ -1869,7 +1870,7 @@
       <c r="AI18" s="17"/>
       <c r="AJ18" s="3"/>
     </row>
-    <row r="19" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A19" s="3"/>
       <c r="B19" s="22"/>
       <c r="C19" s="17"/>
@@ -1907,7 +1908,7 @@
       <c r="AI19" s="17"/>
       <c r="AJ19" s="3"/>
     </row>
-    <row r="20" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A20" s="3"/>
       <c r="B20" s="22"/>
       <c r="C20" s="17"/>
@@ -1945,7 +1946,7 @@
       <c r="AI20" s="17"/>
       <c r="AJ20" s="3"/>
     </row>
-    <row r="21" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A21" s="3"/>
       <c r="B21" s="22"/>
       <c r="C21" s="17"/>
@@ -1983,7 +1984,7 @@
       <c r="AI21" s="17"/>
       <c r="AJ21" s="3"/>
     </row>
-    <row r="22" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A22" s="3"/>
       <c r="B22" s="22"/>
       <c r="C22" s="17"/>
@@ -2021,7 +2022,7 @@
       <c r="AI22" s="17"/>
       <c r="AJ22" s="3"/>
     </row>
-    <row r="23" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A23" s="3"/>
       <c r="B23" s="22"/>
       <c r="C23" s="17"/>
@@ -2059,7 +2060,7 @@
       <c r="AI23" s="17"/>
       <c r="AJ23" s="3"/>
     </row>
-    <row r="24" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A24" s="3"/>
       <c r="B24" s="22"/>
       <c r="C24" s="17"/>
@@ -2097,7 +2098,7 @@
       <c r="AI24" s="17"/>
       <c r="AJ24" s="3"/>
     </row>
-    <row r="25" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A25" s="3"/>
       <c r="B25" s="22"/>
       <c r="C25" s="17"/>
@@ -2135,7 +2136,7 @@
       <c r="AI25" s="17"/>
       <c r="AJ25" s="3"/>
     </row>
-    <row r="26" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A26" s="3"/>
       <c r="B26" s="22"/>
       <c r="C26" s="17"/>
@@ -2173,7 +2174,7 @@
       <c r="AI26" s="17"/>
       <c r="AJ26" s="3"/>
     </row>
-    <row r="27" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A27" s="3"/>
       <c r="B27" s="22"/>
       <c r="C27" s="17"/>
@@ -2211,7 +2212,7 @@
       <c r="AI27" s="17"/>
       <c r="AJ27" s="3"/>
     </row>
-    <row r="28" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A28" s="3"/>
       <c r="B28" s="22"/>
       <c r="C28" s="17"/>
@@ -2249,7 +2250,7 @@
       <c r="AI28" s="17"/>
       <c r="AJ28" s="3"/>
     </row>
-    <row r="29" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A29" s="3"/>
       <c r="B29" s="22"/>
       <c r="C29" s="17"/>
@@ -2287,7 +2288,7 @@
       <c r="AI29" s="17"/>
       <c r="AJ29" s="3"/>
     </row>
-    <row r="30" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A30" s="3"/>
       <c r="B30" s="22"/>
       <c r="C30" s="17"/>
@@ -2325,7 +2326,7 @@
       <c r="AI30" s="17"/>
       <c r="AJ30" s="3"/>
     </row>
-    <row r="31" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A31" s="3"/>
       <c r="B31" s="22"/>
       <c r="C31" s="17"/>
@@ -2363,7 +2364,7 @@
       <c r="AI31" s="17"/>
       <c r="AJ31" s="3"/>
     </row>
-    <row r="32" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A32" s="3"/>
       <c r="B32" s="22"/>
       <c r="C32" s="17"/>
@@ -2401,7 +2402,7 @@
       <c r="AI32" s="17"/>
       <c r="AJ32" s="3"/>
     </row>
-    <row r="33" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A33" s="3"/>
       <c r="B33" s="22"/>
       <c r="C33" s="17"/>
@@ -2439,7 +2440,7 @@
       <c r="AI33" s="17"/>
       <c r="AJ33" s="3"/>
     </row>
-    <row r="34" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A34" s="3"/>
       <c r="B34" s="22"/>
       <c r="C34" s="17"/>
@@ -2477,420 +2478,413 @@
       <c r="AI34" s="17"/>
       <c r="AJ34" s="3"/>
     </row>
-    <row r="35" spans="1:36" s="7" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="27" t="str">
-        <f>"Cantidad Cortes "&amp;B3&amp;":"&amp;CHAR(10)&amp;COUNT(B4:B34)</f>
-        <v>Cantidad Cortes Ciro:
-0</v>
-      </c>
-      <c r="B35" s="27"/>
-      <c r="C35" s="27"/>
+    <row r="35" spans="1:36" s="7" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="33" t="str">
+        <f>"Cantidad Cortes "&amp;B3&amp;": "&amp;COUNT(B4:B34)</f>
+        <v>Cantidad Cortes Barbero1: 0</v>
+      </c>
+      <c r="B35" s="33"/>
+      <c r="C35" s="33"/>
       <c r="D35" s="8"/>
-      <c r="E35" s="27" t="str">
-        <f>"Cantidad Cortes "&amp;F3&amp;":"&amp;CHAR(10)&amp;COUNT(F4:F34)</f>
-        <v>Cantidad Cortes Valentin:
-0</v>
-      </c>
-      <c r="F35" s="27"/>
-      <c r="G35" s="27"/>
+      <c r="E35" s="33" t="str">
+        <f>"Cantidad Cortes "&amp;F3&amp;": "&amp;COUNT(F4:F34)</f>
+        <v>Cantidad Cortes Barbero2: 0</v>
+      </c>
+      <c r="F35" s="33"/>
+      <c r="G35" s="33"/>
       <c r="H35" s="8"/>
-      <c r="I35" s="27" t="str">
-        <f>"Cantidad Cortes "&amp;J3&amp;":"&amp;CHAR(10)&amp;COUNT(J4:J34)</f>
-        <v>Cantidad Cortes Joel:
-0</v>
-      </c>
-      <c r="J35" s="27"/>
-      <c r="K35" s="27"/>
+      <c r="I35" s="33" t="str">
+        <f>"Cantidad Cortes "&amp;J3&amp;": "&amp;COUNT(J4:J34)</f>
+        <v>Cantidad Cortes Barbero3: 0</v>
+      </c>
+      <c r="J35" s="33"/>
+      <c r="K35" s="33"/>
       <c r="L35" s="8"/>
-      <c r="M35" s="27" t="str">
-        <f>"Cantidad Cortes "&amp;N3&amp;":"&amp;CHAR(10)&amp;COUNT(N4:N34)</f>
-        <v>Cantidad Cortes Braian:
-0</v>
-      </c>
-      <c r="N35" s="27"/>
-      <c r="O35" s="27"/>
+      <c r="M35" s="33" t="str">
+        <f>"Cantidad Cortes "&amp;N3&amp;": "&amp;COUNT(N4:N34)</f>
+        <v>Cantidad Cortes Barbero4: 0</v>
+      </c>
+      <c r="N35" s="33"/>
+      <c r="O35" s="33"/>
       <c r="P35" s="8"/>
-      <c r="Q35" s="27" t="str">
-        <f>"Cantidad Cortes "&amp;R3&amp;":"&amp;CHAR(10)&amp;COUNT(R4:R34)</f>
-        <v>Cantidad Cortes Fabricio:
-0</v>
-      </c>
-      <c r="R35" s="27"/>
-      <c r="S35" s="27"/>
+      <c r="Q35" s="33" t="str">
+        <f>"Cantidad Cortes "&amp;R3&amp;": "&amp;COUNT(R4:R34)</f>
+        <v>Cantidad Cortes Barbero5: 0</v>
+      </c>
+      <c r="R35" s="33"/>
+      <c r="S35" s="33"/>
       <c r="T35" s="8"/>
-      <c r="U35" s="27" t="str">
-        <f>"Cantidad Cortes "&amp;V3&amp;":"&amp;CHAR(10)&amp;COUNT(V4:V34)</f>
-        <v>Cantidad Cortes Julian:
-0</v>
-      </c>
-      <c r="V35" s="27"/>
-      <c r="W35" s="27"/>
+      <c r="U35" s="33" t="str">
+        <f>"Cantidad Cortes "&amp;V3&amp;": "&amp;COUNT(V4:V34)</f>
+        <v>Cantidad Cortes Barbero6: 0</v>
+      </c>
+      <c r="V35" s="33"/>
+      <c r="W35" s="33"/>
       <c r="X35" s="8"/>
-      <c r="Y35" s="27" t="str">
-        <f>"Cantidad Cortes "&amp;Z3&amp;":"&amp;CHAR(10)&amp;COUNT(Z4:Z34)</f>
-        <v>Cantidad Cortes Bautista:
-0</v>
-      </c>
-      <c r="Z35" s="27"/>
-      <c r="AA35" s="27"/>
+      <c r="Y35" s="33" t="str">
+        <f>"Cantidad Cortes "&amp;Z3&amp;": "&amp;COUNT(Z4:Z34)</f>
+        <v>Cantidad Cortes Barbero7: 0</v>
+      </c>
+      <c r="Z35" s="33"/>
+      <c r="AA35" s="33"/>
       <c r="AB35" s="8"/>
-      <c r="AC35" s="27" t="str">
-        <f>"Cantidad Cortes "&amp;AD3&amp;":"&amp;CHAR(10)&amp;COUNT(AD4:AD34)</f>
-        <v>Cantidad Cortes Matias:
-0</v>
-      </c>
-      <c r="AD35" s="27"/>
-      <c r="AE35" s="27"/>
+      <c r="AC35" s="33" t="str">
+        <f>"Cantidad Cortes "&amp;AD3&amp;": "&amp;COUNT(AD4:AD34)</f>
+        <v>Cantidad Cortes Barbero8: 0</v>
+      </c>
+      <c r="AD35" s="33"/>
+      <c r="AE35" s="33"/>
       <c r="AF35" s="8"/>
-      <c r="AG35" s="27" t="str">
-        <f>"Cantidad Cortes "&amp;AH3&amp;":"&amp;CHAR(10)&amp;COUNT(AH4:AH34)</f>
-        <v>Cantidad Cortes Barbero9:
-0</v>
-      </c>
-      <c r="AH35" s="27"/>
-      <c r="AI35" s="27"/>
+      <c r="AG35" s="33" t="str">
+        <f>"Cantidad Cortes "&amp;AH3&amp;": "&amp;COUNT(AH4:AH34)</f>
+        <v>Cantidad Cortes Barbero9: 0</v>
+      </c>
+      <c r="AH35" s="33"/>
+      <c r="AI35" s="33"/>
       <c r="AJ35" s="8"/>
     </row>
-    <row r="36" spans="1:36" s="7" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="31" t="str">
-        <f>"Total Cortes "&amp;B3&amp;":"&amp;CHAR(10)&amp;TEXT(INT(SUM(B4:B34)*($M$1/100)),"$#.##0")</f>
-        <v>Total Cortes Ciro:
-$0</v>
-      </c>
-      <c r="B36" s="32"/>
-      <c r="C36" s="33"/>
+    <row r="36" spans="1:36" s="7" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="30" t="str">
+        <f>"Total Cortes "&amp;B3&amp;":"&amp;TEXT(INT(SUM(B4:B34)*($M$1/100)),"$#.##0")</f>
+        <v>Total Cortes Barbero1:$0</v>
+      </c>
+      <c r="B36" s="31"/>
+      <c r="C36" s="32"/>
       <c r="D36" s="8"/>
-      <c r="E36" s="31" t="str">
-        <f>"Total Cortes "&amp;F3&amp;":"&amp;CHAR(10)&amp;TEXT(INT(SUM(F4:F34)*$M$1/100),"$#.##0")</f>
-        <v>Total Cortes Valentin:
-$0</v>
-      </c>
-      <c r="F36" s="32"/>
-      <c r="G36" s="33"/>
+      <c r="E36" s="30" t="str">
+        <f>"Total Cortes "&amp;F3&amp;":"&amp;TEXT(INT(SUM(F4:F34)*$M$1/100),"$#.##0")</f>
+        <v>Total Cortes Barbero2:$0</v>
+      </c>
+      <c r="F36" s="31"/>
+      <c r="G36" s="32"/>
       <c r="H36" s="8"/>
-      <c r="I36" s="31" t="str">
-        <f>"Total Cortes "&amp;J3&amp;":"&amp;CHAR(10)&amp;TEXT(INT(SUM(J4:J34)*$M$1/100),"$#.##0")</f>
-        <v>Total Cortes Joel:
-$0</v>
-      </c>
-      <c r="J36" s="32"/>
-      <c r="K36" s="33"/>
+      <c r="I36" s="30" t="str">
+        <f>"Total Cortes "&amp;J3&amp;":"&amp;TEXT(INT(SUM(J4:J34)*$M$1/100),"$#.##0")</f>
+        <v>Total Cortes Barbero3:$0</v>
+      </c>
+      <c r="J36" s="31"/>
+      <c r="K36" s="32"/>
       <c r="L36" s="8"/>
-      <c r="M36" s="31" t="str">
-        <f>"Total Cortes "&amp;N3&amp;":"&amp;CHAR(10)&amp;TEXT(INT(SUM(N4:N34)*$M$1/100),"$#.##0")</f>
-        <v>Total Cortes Braian:
-$0</v>
-      </c>
-      <c r="N36" s="32"/>
-      <c r="O36" s="33"/>
+      <c r="M36" s="30" t="str">
+        <f>"Total Cortes "&amp;N3&amp;":"&amp;TEXT(INT(SUM(N4:N34)*$M$1/100),"$#.##0")</f>
+        <v>Total Cortes Barbero4:$0</v>
+      </c>
+      <c r="N36" s="31"/>
+      <c r="O36" s="32"/>
       <c r="P36" s="8"/>
-      <c r="Q36" s="31" t="str">
-        <f>"Total Cortes "&amp;R3&amp;":"&amp;CHAR(10)&amp;TEXT(INT(SUM(R4:R34)*$M$1/100),"$#.##0")</f>
-        <v>Total Cortes Fabricio:
-$0</v>
-      </c>
-      <c r="R36" s="32"/>
-      <c r="S36" s="33"/>
+      <c r="Q36" s="30" t="str">
+        <f>"Total Cortes "&amp;R3&amp;":"&amp;TEXT(INT(SUM(R4:R34)*$M$1/100),"$#.##0")</f>
+        <v>Total Cortes Barbero5:$0</v>
+      </c>
+      <c r="R36" s="31"/>
+      <c r="S36" s="32"/>
       <c r="T36" s="8"/>
-      <c r="U36" s="31" t="str">
-        <f>"Total Cortes "&amp;V3&amp;":"&amp;CHAR(10)&amp;TEXT(INT(SUM(V4:V34)*$M$1/100),"$#.##0")</f>
-        <v>Total Cortes Julian:
-$0</v>
-      </c>
-      <c r="V36" s="32"/>
-      <c r="W36" s="33"/>
+      <c r="U36" s="30" t="str">
+        <f>"Total Cortes "&amp;V3&amp;":"&amp;TEXT(INT(SUM(V4:V34)*$M$1/100),"$#.##0")</f>
+        <v>Total Cortes Barbero6:$0</v>
+      </c>
+      <c r="V36" s="31"/>
+      <c r="W36" s="32"/>
       <c r="X36" s="8"/>
-      <c r="Y36" s="31" t="str">
-        <f>"Total Cortes "&amp;Z3&amp;":"&amp;CHAR(10)&amp;TEXT(INT(SUM(Z4:Z34)*$M$1/100),"$#.##0")</f>
-        <v>Total Cortes Bautista:
-$0</v>
-      </c>
-      <c r="Z36" s="32"/>
-      <c r="AA36" s="33"/>
+      <c r="Y36" s="30" t="str">
+        <f>"Total Cortes "&amp;Z3&amp;":"&amp;TEXT(INT(SUM(Z4:Z34)*$M$1/100),"$#.##0")</f>
+        <v>Total Cortes Barbero7:$0</v>
+      </c>
+      <c r="Z36" s="31"/>
+      <c r="AA36" s="32"/>
       <c r="AB36" s="8"/>
-      <c r="AC36" s="31" t="str">
-        <f>"Total Cortes "&amp;AD3&amp;":"&amp;CHAR(10)&amp;TEXT(INT(SUM(AD4:AD34)*$M$1/100),"$#.##0")</f>
-        <v>Total Cortes Matias:
-$0</v>
-      </c>
-      <c r="AD36" s="32"/>
-      <c r="AE36" s="33"/>
+      <c r="AC36" s="30" t="str">
+        <f>"Total Cortes "&amp;AD3&amp;":"&amp;TEXT(INT(SUM(AD4:AD34)*$M$1/100),"$#.##0")</f>
+        <v>Total Cortes Barbero8:$0</v>
+      </c>
+      <c r="AD36" s="31"/>
+      <c r="AE36" s="32"/>
       <c r="AF36" s="8"/>
-      <c r="AG36" s="31" t="str">
-        <f>"Total Cortes "&amp;AH3&amp;":"&amp;CHAR(10)&amp;TEXT(INT(SUM(AH4:AH34)*$M$1/100),"$#.##0")</f>
-        <v>Total Cortes Barbero9:
-$0</v>
-      </c>
-      <c r="AH36" s="32"/>
-      <c r="AI36" s="33"/>
+      <c r="AG36" s="30" t="str">
+        <f>"Total Cortes "&amp;AH3&amp;":"&amp;TEXT(INT(SUM(AH4:AH34)*$M$1/100),"$#.##0")</f>
+        <v>Total Cortes Barbero9:$0</v>
+      </c>
+      <c r="AH36" s="31"/>
+      <c r="AI36" s="32"/>
       <c r="AJ36" s="8"/>
     </row>
-    <row r="37" spans="1:36" s="7" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="27" t="str">
-        <f>"Total Propinas "&amp;B3&amp;":"&amp;CHAR(10)&amp;TEXT(SUM(C4:C34),"$#.##0")</f>
-        <v>Total Propinas Ciro:
-$0</v>
-      </c>
-      <c r="B37" s="27"/>
-      <c r="C37" s="27"/>
+    <row r="37" spans="1:36" s="7" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="33" t="str">
+        <f>"Total Propinas "&amp;B3&amp;":"&amp;TEXT(SUM(C4:C34),"$#.##0")</f>
+        <v>Total Propinas Barbero1:$0</v>
+      </c>
+      <c r="B37" s="33"/>
+      <c r="C37" s="33"/>
       <c r="D37" s="8"/>
-      <c r="E37" s="27" t="str">
-        <f>"Total Propinas "&amp;F3&amp;":"&amp;CHAR(10)&amp;TEXT(SUM(G4:G34),"$#.##0")</f>
-        <v>Total Propinas Valentin:
-$0</v>
-      </c>
-      <c r="F37" s="27"/>
-      <c r="G37" s="27"/>
+      <c r="E37" s="33" t="str">
+        <f>"Total Propinas "&amp;F3&amp;":"&amp;TEXT(SUM(G4:G34),"$#.##0")</f>
+        <v>Total Propinas Barbero2:$0</v>
+      </c>
+      <c r="F37" s="33"/>
+      <c r="G37" s="33"/>
       <c r="H37" s="8"/>
-      <c r="I37" s="27" t="str">
-        <f>"Total Propinas "&amp;J3&amp;":"&amp;CHAR(10)&amp;TEXT(SUM(K4:K34),"$#.##0")</f>
-        <v>Total Propinas Joel:
-$0</v>
-      </c>
-      <c r="J37" s="27"/>
-      <c r="K37" s="27"/>
+      <c r="I37" s="33" t="str">
+        <f>"Total Propinas "&amp;J3&amp;":"&amp;TEXT(SUM(K4:K34),"$#.##0")</f>
+        <v>Total Propinas Barbero3:$0</v>
+      </c>
+      <c r="J37" s="33"/>
+      <c r="K37" s="33"/>
       <c r="L37" s="8"/>
-      <c r="M37" s="27" t="str">
-        <f>"Total Propinas "&amp;N3&amp;":"&amp;CHAR(10)&amp;TEXT(SUM(O4:O34),"$#.##0")</f>
-        <v>Total Propinas Braian:
-$0</v>
-      </c>
-      <c r="N37" s="27"/>
-      <c r="O37" s="27"/>
+      <c r="M37" s="33" t="str">
+        <f>"Total Propinas "&amp;N3&amp;":"&amp;TEXT(SUM(O4:O34),"$#.##0")</f>
+        <v>Total Propinas Barbero4:$0</v>
+      </c>
+      <c r="N37" s="33"/>
+      <c r="O37" s="33"/>
       <c r="P37" s="8"/>
-      <c r="Q37" s="27" t="str">
-        <f>"Total Propinas "&amp;R3&amp;":"&amp;CHAR(10)&amp;TEXT(SUM(S4:S34),"$#.##0")</f>
-        <v>Total Propinas Fabricio:
-$0</v>
-      </c>
-      <c r="R37" s="27"/>
-      <c r="S37" s="27"/>
+      <c r="Q37" s="33" t="str">
+        <f>"Total Propinas "&amp;R3&amp;":"&amp;TEXT(SUM(S4:S34),"$#.##0")</f>
+        <v>Total Propinas Barbero5:$0</v>
+      </c>
+      <c r="R37" s="33"/>
+      <c r="S37" s="33"/>
       <c r="T37" s="8"/>
-      <c r="U37" s="27" t="str">
-        <f>"Total Propinas "&amp;V3&amp;":"&amp;CHAR(10)&amp;TEXT(SUM(W4:W34),"$#.##0")</f>
-        <v>Total Propinas Julian:
-$0</v>
-      </c>
-      <c r="V37" s="27"/>
-      <c r="W37" s="27"/>
+      <c r="U37" s="33" t="str">
+        <f>"Total Propinas "&amp;V3&amp;":"&amp;TEXT(SUM(W4:W34),"$#.##0")</f>
+        <v>Total Propinas Barbero6:$0</v>
+      </c>
+      <c r="V37" s="33"/>
+      <c r="W37" s="33"/>
       <c r="X37" s="8"/>
-      <c r="Y37" s="27" t="str">
-        <f>"Total Propinas "&amp;Z3&amp;":"&amp;CHAR(10)&amp;TEXT(SUM(AA4:AA34),"$#.##0")</f>
-        <v>Total Propinas Bautista:
-$0</v>
-      </c>
-      <c r="Z37" s="27"/>
-      <c r="AA37" s="27"/>
+      <c r="Y37" s="33" t="str">
+        <f>"Total Propinas "&amp;Z3&amp;":"&amp;TEXT(SUM(AA4:AA34),"$#.##0")</f>
+        <v>Total Propinas Barbero7:$0</v>
+      </c>
+      <c r="Z37" s="33"/>
+      <c r="AA37" s="33"/>
       <c r="AB37" s="8"/>
-      <c r="AC37" s="27" t="str">
-        <f>"Total Propinas "&amp;AD3&amp;":"&amp;CHAR(10)&amp;TEXT(SUM(AE4:AE34),"$#.##0")</f>
-        <v>Total Propinas Matias:
-$0</v>
-      </c>
-      <c r="AD37" s="27"/>
-      <c r="AE37" s="27"/>
+      <c r="AC37" s="33" t="str">
+        <f>"Total Propinas "&amp;AD3&amp;":"&amp;TEXT(SUM(AE4:AE34),"$#.##0")</f>
+        <v>Total Propinas Barbero8:$0</v>
+      </c>
+      <c r="AD37" s="33"/>
+      <c r="AE37" s="33"/>
       <c r="AF37" s="8"/>
-      <c r="AG37" s="27" t="str">
-        <f>"Total Propinas "&amp;AH3&amp;":"&amp;CHAR(10)&amp;TEXT(SUM(AI4:AI34),"$#.##0")</f>
-        <v>Total Propinas Barbero9:
-$0</v>
-      </c>
-      <c r="AH37" s="27"/>
-      <c r="AI37" s="27"/>
+      <c r="AG37" s="33" t="str">
+        <f>"Total Propinas "&amp;AH3&amp;":"&amp;TEXT(SUM(AI4:AI34),"$#.##0")</f>
+        <v>Total Propinas Barbero9:$0</v>
+      </c>
+      <c r="AH37" s="33"/>
+      <c r="AI37" s="33"/>
       <c r="AJ37" s="8"/>
     </row>
-    <row r="38" spans="1:36" s="7" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:36" s="7" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="34" t="str">
-        <f>"Adelanto "&amp;B$3&amp;":"&amp;CHAR(10)&amp;TEXT(SUMIF(AdelantosVentas!$A$21:$A$35,"="&amp;B$3,AdelantosVentas!$B$21:$B$35),"$#.##0")</f>
-        <v>Adelanto Ciro:
-$0</v>
+        <f>"Adelanto "&amp;B$3&amp;":"&amp;TEXT(SUMIF(AdelantosVentas!$A$21:$A$35,"="&amp;B$3,AdelantosVentas!$B$21:$B$35),"$#.##0")</f>
+        <v>Adelanto Barbero1:$0</v>
       </c>
       <c r="B38" s="34"/>
       <c r="C38" s="34"/>
       <c r="D38" s="8"/>
       <c r="E38" s="34" t="str">
-        <f>"Adelanto "&amp;F$3&amp;":"&amp;CHAR(10)&amp;TEXT(SUMIF(AdelantosVentas!$A$21:$A$35,"="&amp;F$3,AdelantosVentas!$B$21:$B$35),"$#.##0")</f>
-        <v>Adelanto Valentin:
-$0</v>
+        <f>"Adelanto "&amp;F$3&amp;":"&amp;TEXT(SUMIF(AdelantosVentas!$A$21:$A$35,"="&amp;F$3,AdelantosVentas!$B$21:$B$35),"$#.##0")</f>
+        <v>Adelanto Barbero2:$0</v>
       </c>
       <c r="F38" s="34"/>
       <c r="G38" s="34"/>
       <c r="H38" s="8"/>
       <c r="I38" s="34" t="str">
-        <f>"Adelanto "&amp;J$3&amp;":"&amp;CHAR(10)&amp;TEXT(SUMIF(AdelantosVentas!$A$21:$A$35,"="&amp;J$3,AdelantosVentas!$B$21:$B$35),"$#.##0")</f>
-        <v>Adelanto Joel:
-$0</v>
+        <f>"Adelanto "&amp;J$3&amp;":"&amp;TEXT(SUMIF(AdelantosVentas!$A$21:$A$35,"="&amp;J$3,AdelantosVentas!$B$21:$B$35),"$#.##0")</f>
+        <v>Adelanto Barbero3:$0</v>
       </c>
       <c r="J38" s="34"/>
       <c r="K38" s="34"/>
       <c r="L38" s="8"/>
       <c r="M38" s="34" t="str">
-        <f>"Adelanto "&amp;N$3&amp;":"&amp;CHAR(10)&amp;TEXT(SUMIF(AdelantosVentas!$A$21:$A$35,"="&amp;N$3,AdelantosVentas!$B$21:$B$35),"$#.##0")</f>
-        <v>Adelanto Braian:
-$0</v>
+        <f>"Adelanto "&amp;N$3&amp;":"&amp;TEXT(SUMIF(AdelantosVentas!$A$21:$A$35,"="&amp;N$3,AdelantosVentas!$B$21:$B$35),"$#.##0")</f>
+        <v>Adelanto Barbero4:$0</v>
       </c>
       <c r="N38" s="34"/>
       <c r="O38" s="34"/>
       <c r="P38" s="8"/>
       <c r="Q38" s="34" t="str">
-        <f>"Adelanto "&amp;R$3&amp;":"&amp;CHAR(10)&amp;TEXT(SUMIF(AdelantosVentas!$A$21:$A$35,"="&amp;R$3,AdelantosVentas!$B$21:$B$35),"$#.##0")</f>
-        <v>Adelanto Fabricio:
-$0</v>
+        <f>"Adelanto "&amp;R$3&amp;":"&amp;TEXT(SUMIF(AdelantosVentas!$A$21:$A$35,"="&amp;R$3,AdelantosVentas!$B$21:$B$35),"$#.##0")</f>
+        <v>Adelanto Barbero5:$0</v>
       </c>
       <c r="R38" s="34"/>
       <c r="S38" s="34"/>
       <c r="T38" s="8"/>
       <c r="U38" s="34" t="str">
-        <f>"Adelanto "&amp;V$3&amp;":"&amp;CHAR(10)&amp;TEXT(SUMIF(AdelantosVentas!$A$21:$A$35,"="&amp;V$3,AdelantosVentas!$B$21:$B$35),"$#.##0")</f>
-        <v>Adelanto Julian:
-$0</v>
+        <f>"Adelanto "&amp;V$3&amp;":"&amp;TEXT(SUMIF(AdelantosVentas!$A$21:$A$35,"="&amp;V$3,AdelantosVentas!$B$21:$B$35),"$#.##0")</f>
+        <v>Adelanto Barbero6:$0</v>
       </c>
       <c r="V38" s="34"/>
       <c r="W38" s="34"/>
       <c r="X38" s="8"/>
       <c r="Y38" s="34" t="str">
-        <f>"Adelanto "&amp;Z$3&amp;":"&amp;CHAR(10)&amp;TEXT(SUMIF(AdelantosVentas!$A$21:$A$35,"="&amp;Z$3,AdelantosVentas!$B$21:$B$35),"$#.##0")</f>
-        <v>Adelanto Bautista:
-$0</v>
+        <f>"Adelanto "&amp;Z$3&amp;":"&amp;TEXT(SUMIF(AdelantosVentas!$A$21:$A$35,"="&amp;Z$3,AdelantosVentas!$B$21:$B$35),"$#.##0")</f>
+        <v>Adelanto Barbero7:$0</v>
       </c>
       <c r="Z38" s="34"/>
       <c r="AA38" s="34"/>
       <c r="AB38" s="8"/>
       <c r="AC38" s="34" t="str">
-        <f>"Adelanto "&amp;AD$3&amp;":"&amp;CHAR(10)&amp;TEXT(SUMIF(AdelantosVentas!$A$21:$A$35,"="&amp;AD$3,AdelantosVentas!$B$21:$B$35),"$#.##0")</f>
-        <v>Adelanto Matias:
-$0</v>
+        <f>"Adelanto "&amp;AD$3&amp;":"&amp;TEXT(SUMIF(AdelantosVentas!$A$21:$A$35,"="&amp;AD$3,AdelantosVentas!$B$21:$B$35),"$#.##0")</f>
+        <v>Adelanto Barbero8:$0</v>
       </c>
       <c r="AD38" s="34"/>
       <c r="AE38" s="34"/>
       <c r="AF38" s="8"/>
       <c r="AG38" s="34" t="str">
-        <f>"Adelanto "&amp;AH$3&amp;":"&amp;CHAR(10)&amp;TEXT(SUMIF(AdelantosVentas!$A$21:$A$35,"="&amp;AH$3,AdelantosVentas!$B$21:$B$35),"$#.##0")</f>
-        <v>Adelanto Barbero9:
-$0</v>
+        <f>"Adelanto "&amp;AH$3&amp;":"&amp;TEXT(SUMIF(AdelantosVentas!$A$21:$A$35,"="&amp;AH$3,AdelantosVentas!$B$21:$B$35),"$#.##0")</f>
+        <v>Adelanto Barbero9:$0</v>
       </c>
       <c r="AH38" s="34"/>
       <c r="AI38" s="34"/>
       <c r="AJ38" s="8"/>
     </row>
-    <row r="39" spans="1:36" s="7" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="27" t="str">
-        <f>"Total "&amp;B$3&amp;":"&amp;CHAR(10)&amp;TEXT(VALUE(INT(SUM(B4:B34)*$M$1/100)+SUM(C4:C34)-SUMIF(AdelantosVentas!$A$21:$A$35,"="&amp;B$3,AdelantosVentas!$B$21:$B$35)),"$#.##0")</f>
-        <v>Total Ciro:
-$0</v>
-      </c>
-      <c r="B39" s="27"/>
-      <c r="C39" s="27"/>
+    <row r="39" spans="1:36" s="7" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="33" t="str">
+        <f>"Total "&amp;B$3&amp;":"&amp;TEXT(VALUE(INT(SUM(B4:B34)*$M$1/100)+SUM(C4:C34)-SUMIF(AdelantosVentas!$A$21:$A$35,"="&amp;B$3,AdelantosVentas!$B$21:$B$35)),"$#.##0")</f>
+        <v>Total Barbero1:$0</v>
+      </c>
+      <c r="B39" s="33"/>
+      <c r="C39" s="33"/>
       <c r="D39" s="23"/>
-      <c r="E39" s="27" t="str">
-        <f>"Total "&amp;F$3&amp;":"&amp;CHAR(10)&amp;TEXT(VALUE(INT(SUM(F4:F34)*$M$1/100)+SUM(G4:G34)-SUMIF(AdelantosVentas!$A$21:$A$35,"="&amp;F$3,AdelantosVentas!$B$21:$B$35)),"$#.##0")</f>
-        <v>Total Valentin:
-$0</v>
-      </c>
-      <c r="F39" s="27"/>
-      <c r="G39" s="27"/>
+      <c r="E39" s="33" t="str">
+        <f>"Total "&amp;F$3&amp;":"&amp;TEXT(VALUE(INT(SUM(F4:F34)*$M$1/100)+SUM(G4:G34)-SUMIF(AdelantosVentas!$A$21:$A$35,"="&amp;F$3,AdelantosVentas!$B$21:$B$35)),"$#.##0")</f>
+        <v>Total Barbero2:$0</v>
+      </c>
+      <c r="F39" s="33"/>
+      <c r="G39" s="33"/>
       <c r="H39" s="23"/>
-      <c r="I39" s="27" t="str">
-        <f>"Total "&amp;J$3&amp;":"&amp;CHAR(10)&amp;TEXT(VALUE(INT(SUM(J4:J34)*$M$1/100)+SUM(K4:K34)-SUMIF(AdelantosVentas!$A$21:$A$35,"="&amp;J$3,AdelantosVentas!$B$21:$B$35)),"$#.##0")</f>
-        <v>Total Joel:
-$0</v>
-      </c>
-      <c r="J39" s="27"/>
-      <c r="K39" s="27"/>
+      <c r="I39" s="33" t="str">
+        <f>"Total "&amp;J$3&amp;":"&amp;TEXT(VALUE(INT(SUM(J4:J34)*$M$1/100)+SUM(K4:K34)-SUMIF(AdelantosVentas!$A$21:$A$35,"="&amp;J$3,AdelantosVentas!$B$21:$B$35)),"$#.##0")</f>
+        <v>Total Barbero3:$0</v>
+      </c>
+      <c r="J39" s="33"/>
+      <c r="K39" s="33"/>
       <c r="L39" s="23"/>
-      <c r="M39" s="27" t="str">
-        <f>"Total "&amp;N$3&amp;":"&amp;CHAR(10)&amp;TEXT(VALUE(INT(SUM(N4:N34)*$M$1/100)+SUM(O4:O34)-SUMIF(AdelantosVentas!$A$21:$A$35,"="&amp;N$3,AdelantosVentas!$B$21:$B$35)),"$#.##0")</f>
-        <v>Total Braian:
-$0</v>
-      </c>
-      <c r="N39" s="27"/>
-      <c r="O39" s="27"/>
+      <c r="M39" s="33" t="str">
+        <f>"Total "&amp;N$3&amp;":"&amp;TEXT(VALUE(INT(SUM(N4:N34)*$M$1/100)+SUM(O4:O34)-SUMIF(AdelantosVentas!$A$21:$A$35,"="&amp;N$3,AdelantosVentas!$B$21:$B$35)),"$#.##0")</f>
+        <v>Total Barbero4:$0</v>
+      </c>
+      <c r="N39" s="33"/>
+      <c r="O39" s="33"/>
       <c r="P39" s="23"/>
-      <c r="Q39" s="28" t="str">
-        <f>"Total "&amp;R$3&amp;":"&amp;CHAR(10)&amp;TEXT(VALUE(INT(SUM(R4:R34)*$M$1/100)+SUM(S4:S34)-SUMIF(AdelantosVentas!$A$21:$A$35,"="&amp;R$3,AdelantosVentas!$B$21:$B$35)),"$#.##0")</f>
-        <v>Total Fabricio:
-$0</v>
-      </c>
-      <c r="R39" s="28"/>
-      <c r="S39" s="27"/>
+      <c r="Q39" s="46" t="str">
+        <f>"Total "&amp;R$3&amp;":"&amp;TEXT(VALUE(INT(SUM(R4:R34)*$M$1/100)+SUM(S4:S34)-SUMIF(AdelantosVentas!$A$21:$A$35,"="&amp;R$3,AdelantosVentas!$B$21:$B$35)),"$#.##0")</f>
+        <v>Total Barbero5:$0</v>
+      </c>
+      <c r="R39" s="46"/>
+      <c r="S39" s="33"/>
       <c r="T39" s="23"/>
-      <c r="U39" s="27" t="str">
-        <f>"Total "&amp;V$3&amp;":"&amp;CHAR(10)&amp;TEXT(VALUE(INT(SUM(V4:V34)*$M$1/100)+SUM(W4:W34)-SUMIF(AdelantosVentas!$A$21:$A$35,"="&amp;V$3,AdelantosVentas!$B$21:$B$35)),"$#.##0")</f>
-        <v>Total Julian:
-$0</v>
-      </c>
-      <c r="V39" s="27"/>
-      <c r="W39" s="27"/>
+      <c r="U39" s="33" t="str">
+        <f>"Total "&amp;V$3&amp;":"&amp;TEXT(VALUE(INT(SUM(V4:V34)*$M$1/100)+SUM(W4:W34)-SUMIF(AdelantosVentas!$A$21:$A$35,"="&amp;V$3,AdelantosVentas!$B$21:$B$35)),"$#.##0")</f>
+        <v>Total Barbero6:$0</v>
+      </c>
+      <c r="V39" s="33"/>
+      <c r="W39" s="33"/>
       <c r="X39" s="23"/>
-      <c r="Y39" s="27" t="str">
-        <f>"Total "&amp;Z$3&amp;":"&amp;CHAR(10)&amp;TEXT(VALUE(INT(SUM(Z4:Z34)*$M$1/100)+SUM(AA4:AA34)-SUMIF(AdelantosVentas!$A$21:$A$35,"="&amp;Z$3,AdelantosVentas!$B$21:$B$35)),"$#.##0")</f>
-        <v>Total Bautista:
-$0</v>
-      </c>
-      <c r="Z39" s="27"/>
-      <c r="AA39" s="27"/>
+      <c r="Y39" s="33" t="str">
+        <f>"Total "&amp;Z$3&amp;":"&amp;TEXT(VALUE(INT(SUM(Z4:Z34)*$M$1/100)+SUM(AA4:AA34)-SUMIF(AdelantosVentas!$A$21:$A$35,"="&amp;Z$3,AdelantosVentas!$B$21:$B$35)),"$#.##0")</f>
+        <v>Total Barbero7:$0</v>
+      </c>
+      <c r="Z39" s="33"/>
+      <c r="AA39" s="33"/>
       <c r="AB39" s="23"/>
-      <c r="AC39" s="27" t="str">
-        <f>"Total "&amp;AD$3&amp;":"&amp;CHAR(10)&amp;TEXT(VALUE(INT(SUM(AD4:AD34)*$M$1/100)+SUM(AE4:AE34)-SUMIF(AdelantosVentas!$A$21:$A$35,"="&amp;AD$3,AdelantosVentas!$B$21:$B$35)),"$#.##0")</f>
-        <v>Total Matias:
-$0</v>
-      </c>
-      <c r="AD39" s="27"/>
-      <c r="AE39" s="27"/>
+      <c r="AC39" s="33" t="str">
+        <f>"Total "&amp;AD$3&amp;":"&amp;TEXT(VALUE(INT(SUM(AD4:AD34)*$M$1/100)+SUM(AE4:AE34)-SUMIF(AdelantosVentas!$A$21:$A$35,"="&amp;AD$3,AdelantosVentas!$B$21:$B$35)),"$#.##0")</f>
+        <v>Total Barbero8:$0</v>
+      </c>
+      <c r="AD39" s="33"/>
+      <c r="AE39" s="33"/>
       <c r="AF39" s="23"/>
-      <c r="AG39" s="27" t="str">
-        <f>"Total "&amp;AH$3&amp;":"&amp;CHAR(10)&amp;TEXT(VALUE(INT(SUM(AH4:AH34)*$M$1/100)+SUM(AI4:AI34)-SUMIF(AdelantosVentas!$A$21:$A$35,"="&amp;AH$3,AdelantosVentas!$B$21:$B$35)),"$#.##0")</f>
-        <v>Total Barbero9:
-$0</v>
-      </c>
-      <c r="AH39" s="27"/>
-      <c r="AI39" s="27"/>
+      <c r="AG39" s="33" t="str">
+        <f>"Total "&amp;AH$3&amp;":"&amp;TEXT(VALUE(INT(SUM(AH4:AH34)*$M$1/100)+SUM(AI4:AI34)-SUMIF(AdelantosVentas!$A$21:$A$35,"="&amp;AH$3,AdelantosVentas!$B$21:$B$35)),"$#.##0")</f>
+        <v>Total Barbero9:$0</v>
+      </c>
+      <c r="AH39" s="33"/>
+      <c r="AI39" s="33"/>
       <c r="AJ39" s="23"/>
     </row>
-    <row r="40" spans="1:36" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B40" s="35" t="str" cm="1">
+    <row r="40" spans="1:36" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B40" s="42" t="str" cm="1">
         <f t="array" ref="B40">"Total Caja: " &amp; TEXT(SUM(_xlfn._xlws.FILTER(B4:B34,ISBLANK(D4:D34)),_xlfn._xlws.FILTER(F4:F34,ISBLANK(H4:H34)),_xlfn._xlws.FILTER(J4:J34,ISBLANK(L4:L34)),_xlfn._xlws.FILTER(N4:N34,ISBLANK(P4:P34)),_xlfn._xlws.FILTER(R4:R34,ISBLANK(T4:T34)),_xlfn._xlws.FILTER(V4:V34,ISBLANK(X4:X34)),_xlfn._xlws.FILTER(Z4:Z34,ISBLANK(AB4:AB34)),_xlfn._xlws.FILTER(AD4:AD34,ISBLANK(AF4:AF34)),_xlfn._xlws.FILTER(AH4:AH34,ISBLANK(AJ4:AJ34)),AdelantosVentas!G36)-AdelantosVentas!B36+SUM(_xlfn._xlws.FILTER(C4:C34,ISBLANK(D4:D34)),_xlfn._xlws.FILTER(G4:G34,ISBLANK(H4:H34)),_xlfn._xlws.FILTER(K4:K34,ISBLANK(L4:L34)),_xlfn._xlws.FILTER(O4:O34,ISBLANK(P4:P34)),_xlfn._xlws.FILTER(S4:S34,ISBLANK(T4:T34)),_xlfn._xlws.FILTER(W4:W34,ISBLANK(X4:X34)),_xlfn._xlws.FILTER(AA4:AA34,ISBLANK(AB4:AB34)),_xlfn._xlws.FILTER(AE4:AE34,ISBLANK(AF4:AF34)),_xlfn._xlws.FILTER(AI4:AI34,ISBLANK(AJ4:AJ34))) + I1,"$#.##0")</f>
         <v>Total Caja: $0</v>
       </c>
-      <c r="C40" s="35"/>
-      <c r="D40" s="35"/>
-      <c r="E40" s="35"/>
-      <c r="F40" s="36" t="str" cm="1">
+      <c r="C40" s="42"/>
+      <c r="D40" s="42"/>
+      <c r="E40" s="42"/>
+      <c r="F40" s="43" t="str" cm="1">
         <f t="array" ref="F40">"Total MP: " &amp; TEXT(SUM(_xlfn._xlws.FILTER(B4:B36,D4:D36="X",0),_xlfn._xlws.FILTER(F4:F34,H4:H34="X",0),_xlfn._xlws.FILTER(J4:J34,L4:L34="X",0),_xlfn._xlws.FILTER(N4:N34,P4:P34="X",0),_xlfn._xlws.FILTER(R4:R34,T4:T34="X",0),_xlfn._xlws.FILTER(V4:V34,X4:X34="X",0),_xlfn._xlws.FILTER(Z4:Z34,AB4:AB34="X",0),_xlfn._xlws.FILTER(AD4:AD34,AF4:AF34="X",0),_xlfn._xlws.FILTER(AH4:AH34,AJ4:AJ34="X",0),AdelantosVentas!H36) + SUM(_xlfn._xlws.FILTER(C4:C36,D4:D36="X",0),_xlfn._xlws.FILTER(G4:G34,H4:H34="X",0),_xlfn._xlws.FILTER(K4:K34,L4:L34="X",0),_xlfn._xlws.FILTER(O4:O34,P4:P34="X",0),_xlfn._xlws.FILTER(S4:S34,T4:T34="X",0),_xlfn._xlws.FILTER(W4:W34,X4:X34="X",0),_xlfn._xlws.FILTER(AA4:AA34,AB4:AB34="X",0),_xlfn._xlws.FILTER(AE4:AE34,AF4:AF34="X",0),_xlfn._xlws.FILTER(AI4:AI34,AJ4:AJ34="X",0))-AdelantosVentas!C36-IF(D39="X",INT(REPLACE(A39,1,8+LEN(B3),"")),0)-IF(H39="X",INT(REPLACE(E39,1,8+LEN(F3),"")),0)-IF(L39="X",INT(REPLACE(I39,1,8+LEN(J3),"")),0)-IF(P39="X",INT(REPLACE(M39,1,8+LEN(N3),"")),0)-IF(T39="X",INT(REPLACE(Q39,1,8+LEN(R3),"")),0)-IF(X39="X",INT(REPLACE(U39,1,8+LEN(V3),"")),0)-IF(AB39="X",INT(REPLACE(Y39,1,8+LEN(Z3),"")),0)-IF(AF39="X",INT(REPLACE(AC39,1,8+LEN(AD3),"")),0)-IF(AJ39="X",INT(REPLACE(AG39,1,8+LEN(H3),"")),0),"$#.##0")</f>
         <v>Total MP: $0</v>
       </c>
-      <c r="G40" s="37"/>
-      <c r="H40" s="37"/>
+      <c r="G40" s="44"/>
+      <c r="H40" s="44"/>
       <c r="I40" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="J40" s="38"/>
-      <c r="K40" s="38"/>
-      <c r="L40" s="38"/>
-      <c r="M40" s="36" t="str">
+        <v>13</v>
+      </c>
+      <c r="J40" s="45"/>
+      <c r="K40" s="45"/>
+      <c r="L40" s="45"/>
+      <c r="M40" s="43" t="str">
         <f>"Cantidad cortes: "&amp;COUNTIF(B4:B36,"&gt;0" )+COUNTIF(F4:F34,"&gt;0" )+COUNTIF(J4:J34,"&gt;0" )+COUNTIF(N4:N34,"&gt;0" )+COUNTIF(R4:R34,"&gt;0" )+COUNTIF(V4:V34,"&gt;0" )+COUNTIF(Z4:Z34,"&gt;0" )+COUNTIF(AD4:AD34,"&gt;0" )+COUNTIF(AH4:AH34,"&gt;0" )&amp;""</f>
         <v>Cantidad cortes: 0</v>
       </c>
-      <c r="N40" s="37"/>
-      <c r="O40" s="37"/>
+      <c r="N40" s="44"/>
+      <c r="O40" s="44"/>
       <c r="P40" s="24" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="Q40" s="25"/>
-      <c r="R40" s="44"/>
-      <c r="S40" s="45"/>
-      <c r="T40" s="45"/>
-      <c r="U40" s="45"/>
-      <c r="V40" s="45"/>
-      <c r="W40" s="45"/>
-      <c r="X40" s="45"/>
-      <c r="Y40" s="45"/>
-      <c r="Z40" s="45"/>
-      <c r="AA40" s="45"/>
-      <c r="AB40" s="46"/>
+      <c r="R40" s="27"/>
+      <c r="S40" s="28"/>
+      <c r="T40" s="28"/>
+      <c r="U40" s="28"/>
+      <c r="V40" s="28"/>
+      <c r="W40" s="28"/>
+      <c r="X40" s="28"/>
+      <c r="Y40" s="28"/>
+      <c r="Z40" s="28"/>
+      <c r="AA40" s="28"/>
+      <c r="AB40" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="54">
+    <mergeCell ref="AG39:AI39"/>
+    <mergeCell ref="M39:O39"/>
+    <mergeCell ref="Q39:S39"/>
+    <mergeCell ref="U39:W39"/>
+    <mergeCell ref="Y39:AA39"/>
+    <mergeCell ref="AC39:AE39"/>
+    <mergeCell ref="Q35:S35"/>
+    <mergeCell ref="U35:W35"/>
+    <mergeCell ref="Y35:AA35"/>
+    <mergeCell ref="AC35:AE35"/>
+    <mergeCell ref="AG35:AI35"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="M36:O36"/>
+    <mergeCell ref="M37:O37"/>
+    <mergeCell ref="M38:O38"/>
+    <mergeCell ref="B40:E40"/>
+    <mergeCell ref="E38:G38"/>
+    <mergeCell ref="F40:H40"/>
+    <mergeCell ref="J40:L40"/>
+    <mergeCell ref="M40:O40"/>
+    <mergeCell ref="A35:C35"/>
+    <mergeCell ref="E35:G35"/>
+    <mergeCell ref="I35:K35"/>
+    <mergeCell ref="M35:O35"/>
+    <mergeCell ref="A39:C39"/>
+    <mergeCell ref="E39:G39"/>
+    <mergeCell ref="I39:K39"/>
+    <mergeCell ref="I36:K36"/>
+    <mergeCell ref="I37:K37"/>
+    <mergeCell ref="I38:K38"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="I1:J1"/>
+    <mergeCell ref="K1:L1"/>
+    <mergeCell ref="A36:C36"/>
+    <mergeCell ref="A37:C37"/>
+    <mergeCell ref="A38:C38"/>
+    <mergeCell ref="E36:G36"/>
+    <mergeCell ref="E37:G37"/>
     <mergeCell ref="R40:AB40"/>
     <mergeCell ref="AC36:AE36"/>
     <mergeCell ref="AC37:AE37"/>
@@ -2907,44 +2901,6 @@
     <mergeCell ref="U37:W37"/>
     <mergeCell ref="Y36:AA36"/>
     <mergeCell ref="Y37:AA37"/>
-    <mergeCell ref="A36:C36"/>
-    <mergeCell ref="A37:C37"/>
-    <mergeCell ref="A38:C38"/>
-    <mergeCell ref="E36:G36"/>
-    <mergeCell ref="E37:G37"/>
-    <mergeCell ref="I36:K36"/>
-    <mergeCell ref="I37:K37"/>
-    <mergeCell ref="I38:K38"/>
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="I1:J1"/>
-    <mergeCell ref="K1:L1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="M36:O36"/>
-    <mergeCell ref="M37:O37"/>
-    <mergeCell ref="M38:O38"/>
-    <mergeCell ref="B40:E40"/>
-    <mergeCell ref="E38:G38"/>
-    <mergeCell ref="F40:H40"/>
-    <mergeCell ref="J40:L40"/>
-    <mergeCell ref="M40:O40"/>
-    <mergeCell ref="A35:C35"/>
-    <mergeCell ref="E35:G35"/>
-    <mergeCell ref="I35:K35"/>
-    <mergeCell ref="M35:O35"/>
-    <mergeCell ref="A39:C39"/>
-    <mergeCell ref="E39:G39"/>
-    <mergeCell ref="I39:K39"/>
-    <mergeCell ref="Q35:S35"/>
-    <mergeCell ref="U35:W35"/>
-    <mergeCell ref="Y35:AA35"/>
-    <mergeCell ref="AC35:AE35"/>
-    <mergeCell ref="AG35:AI35"/>
-    <mergeCell ref="AG39:AI39"/>
-    <mergeCell ref="M39:O39"/>
-    <mergeCell ref="Q39:S39"/>
-    <mergeCell ref="U39:W39"/>
-    <mergeCell ref="Y39:AA39"/>
-    <mergeCell ref="AC39:AE39"/>
   </mergeCells>
   <conditionalFormatting sqref="A39">
     <cfRule type="expression" dxfId="33" priority="42">
@@ -3080,51 +3036,51 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91F4A758-FA64-4BB3-BD95-5A03C71FE753}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:H36"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.21875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="40.7265625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="22.7265625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="11.453125" style="1" customWidth="1"/>
-    <col min="4" max="5" width="9.1796875" style="1"/>
-    <col min="6" max="6" width="28.26953125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="20.26953125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="9.7265625" style="1" customWidth="1"/>
-    <col min="9" max="16384" width="9.1796875" style="1"/>
+    <col min="1" max="1" width="40.77734375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="22.77734375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="11.44140625" style="1" customWidth="1"/>
+    <col min="4" max="5" width="9.21875" style="1"/>
+    <col min="6" max="6" width="28.21875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="20.21875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="9.77734375" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="9.21875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="47" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B1" s="48"/>
       <c r="C1" s="49"/>
       <c r="F1" s="47" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G1" s="48"/>
       <c r="H1" s="49"/>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>6</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>7</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="3"/>
       <c r="B3" s="17"/>
       <c r="C3" s="14"/>
@@ -3132,7 +3088,7 @@
       <c r="G3" s="18"/>
       <c r="H3" s="18"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="3"/>
       <c r="B4" s="17"/>
       <c r="C4" s="14"/>
@@ -3140,7 +3096,7 @@
       <c r="G4" s="18"/>
       <c r="H4" s="18"/>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
       <c r="B5" s="17"/>
       <c r="C5" s="14"/>
@@ -3148,7 +3104,7 @@
       <c r="G5" s="18"/>
       <c r="H5" s="18"/>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="3"/>
       <c r="B6" s="17"/>
       <c r="C6" s="14"/>
@@ -3156,7 +3112,7 @@
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="3"/>
       <c r="B7" s="17"/>
       <c r="C7" s="14"/>
@@ -3164,7 +3120,7 @@
       <c r="G7" s="18"/>
       <c r="H7" s="18"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="3"/>
       <c r="B8" s="17"/>
       <c r="C8" s="14"/>
@@ -3172,7 +3128,7 @@
       <c r="G8" s="18"/>
       <c r="H8" s="18"/>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="3"/>
       <c r="B9" s="17"/>
       <c r="C9" s="14"/>
@@ -3180,7 +3136,7 @@
       <c r="G9" s="18"/>
       <c r="H9" s="18"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="3"/>
       <c r="B10" s="17"/>
       <c r="C10" s="14"/>
@@ -3188,7 +3144,7 @@
       <c r="G10" s="18"/>
       <c r="H10" s="18"/>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="3"/>
       <c r="B11" s="17"/>
       <c r="C11" s="14"/>
@@ -3196,7 +3152,7 @@
       <c r="G11" s="18"/>
       <c r="H11" s="18"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="3"/>
       <c r="B12" s="17"/>
       <c r="C12" s="14"/>
@@ -3204,7 +3160,7 @@
       <c r="G12" s="18"/>
       <c r="H12" s="18"/>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="3"/>
       <c r="B13" s="17"/>
       <c r="C13" s="14"/>
@@ -3212,7 +3168,7 @@
       <c r="G13" s="18"/>
       <c r="H13" s="18"/>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="3"/>
       <c r="B14" s="17"/>
       <c r="C14" s="14"/>
@@ -3220,7 +3176,7 @@
       <c r="G14" s="18"/>
       <c r="H14" s="18"/>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="3"/>
       <c r="B15" s="17"/>
       <c r="C15" s="14"/>
@@ -3228,7 +3184,7 @@
       <c r="G15" s="18"/>
       <c r="H15" s="18"/>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="3"/>
       <c r="B16" s="17"/>
       <c r="C16" s="14"/>
@@ -3236,7 +3192,7 @@
       <c r="G16" s="18"/>
       <c r="H16" s="18"/>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="3"/>
       <c r="B17" s="17"/>
       <c r="C17" s="14"/>
@@ -3244,7 +3200,7 @@
       <c r="G17" s="18"/>
       <c r="H17" s="18"/>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="3"/>
       <c r="B18" s="17"/>
       <c r="C18" s="14"/>
@@ -3252,9 +3208,9 @@
       <c r="G18" s="18"/>
       <c r="H18" s="18"/>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A19" s="50" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B19" s="51"/>
       <c r="C19" s="52"/>
@@ -3262,12 +3218,12 @@
       <c r="G19" s="18"/>
       <c r="H19" s="18"/>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>2</v>
@@ -3276,9 +3232,10 @@
       <c r="G20" s="18"/>
       <c r="H20" s="18"/>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A21" s="3" t="s">
-        <v>18</v>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="str">
+        <f>Barberos!B$3</f>
+        <v>Barbero1</v>
       </c>
       <c r="B21" s="17"/>
       <c r="C21" s="14"/>
@@ -3286,9 +3243,10 @@
       <c r="G21" s="18"/>
       <c r="H21" s="18"/>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A22" s="3" t="s">
-        <v>19</v>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="str">
+        <f>Barberos!F$3</f>
+        <v>Barbero2</v>
       </c>
       <c r="B22" s="17"/>
       <c r="C22" s="14"/>
@@ -3296,9 +3254,10 @@
       <c r="G22" s="18"/>
       <c r="H22" s="18"/>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A23" s="3" t="s">
-        <v>20</v>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="str">
+        <f>Barberos!J$3</f>
+        <v>Barbero3</v>
       </c>
       <c r="B23" s="17"/>
       <c r="C23" s="14"/>
@@ -3306,9 +3265,10 @@
       <c r="G23" s="18"/>
       <c r="H23" s="18"/>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A24" s="3" t="s">
-        <v>22</v>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="str">
+        <f>Barberos!N$3</f>
+        <v>Barbero4</v>
       </c>
       <c r="B24" s="17"/>
       <c r="C24" s="14"/>
@@ -3316,9 +3276,10 @@
       <c r="G24" s="18"/>
       <c r="H24" s="18"/>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A25" s="3" t="s">
-        <v>25</v>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="str">
+        <f>Barberos!R$3</f>
+        <v>Barbero5</v>
       </c>
       <c r="B25" s="17"/>
       <c r="C25" s="14"/>
@@ -3326,9 +3287,10 @@
       <c r="G25" s="18"/>
       <c r="H25" s="18"/>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A26" s="3" t="s">
-        <v>23</v>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" s="3" t="str">
+        <f>Barberos!V$3</f>
+        <v>Barbero6</v>
       </c>
       <c r="B26" s="17"/>
       <c r="C26" s="14"/>
@@ -3336,9 +3298,10 @@
       <c r="G26" s="18"/>
       <c r="H26" s="18"/>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A27" s="3" t="s">
-        <v>26</v>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="str">
+        <f>Barberos!Z$3</f>
+        <v>Barbero7</v>
       </c>
       <c r="B27" s="17"/>
       <c r="C27" s="14"/>
@@ -3346,9 +3309,10 @@
       <c r="G27" s="18"/>
       <c r="H27" s="18"/>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A28" s="3" t="s">
-        <v>21</v>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" s="3" t="str">
+        <f>Barberos!AD$3</f>
+        <v>Barbero8</v>
       </c>
       <c r="B28" s="17"/>
       <c r="C28" s="14"/>
@@ -3356,15 +3320,18 @@
       <c r="G28" s="18"/>
       <c r="H28" s="18"/>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A29" s="3"/>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="str">
+        <f>Barberos!AH$3</f>
+        <v>Barbero9</v>
+      </c>
       <c r="B29" s="17"/>
       <c r="C29" s="14"/>
       <c r="F29" s="14"/>
       <c r="G29" s="18"/>
       <c r="H29" s="18"/>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="3"/>
       <c r="B30" s="17"/>
       <c r="C30" s="14"/>
@@ -3372,7 +3339,7 @@
       <c r="G30" s="18"/>
       <c r="H30" s="18"/>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="3"/>
       <c r="B31" s="17"/>
       <c r="C31" s="14"/>
@@ -3380,7 +3347,7 @@
       <c r="G31" s="18"/>
       <c r="H31" s="18"/>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="3"/>
       <c r="B32" s="17"/>
       <c r="C32" s="14"/>
@@ -3388,7 +3355,7 @@
       <c r="G32" s="18"/>
       <c r="H32" s="18"/>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="3"/>
       <c r="B33" s="17"/>
       <c r="C33" s="14"/>
@@ -3396,7 +3363,7 @@
       <c r="G33" s="18"/>
       <c r="H33" s="18"/>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="3"/>
       <c r="B34" s="17"/>
       <c r="C34" s="14"/>
@@ -3404,25 +3371,25 @@
       <c r="G34" s="18"/>
       <c r="H34" s="18"/>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A35" s="3"/>
       <c r="B35" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C35" s="16" t="s">
         <v>2</v>
       </c>
       <c r="F35" s="14"/>
       <c r="G35" s="19" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H35" s="19" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="26.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:8" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B36" s="18">
         <f>SUMIF(C3:C34,"=",B3:B34)</f>
@@ -3433,7 +3400,7 @@
         <v>0</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G36" s="18">
         <f>SUMIF(H3:H34,"=",G3:G34)</f>

</xml_diff>